<commit_message>
Add sorted, labelled gap table to Calc for the size-of-the-prize chart
Every dashboard chart now has a ready-made formula range on the Calc
sheet; the guide lists them as the fastest route, with two PivotTables
kept to prove the numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MZwMxskGNyzCVskxeKKHE
</commit_message>
<xml_diff>
--- a/buan-b205-dashboard/Team_Dashboard_starter.xlsx
+++ b/buan-b205-dashboard/Team_Dashboard_starter.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7165" uniqueCount="1131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7169" uniqueCount="1134">
   <si>
     <t xml:space="preserve">Build your dashboard on this sheet in Excel (charts, headline, limitation, team names).</t>
   </si>
@@ -3369,7 +3369,16 @@
     <t xml:space="preserve">Sister avg purchase</t>
   </si>
   <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch – weakest line (sorted)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total opportunity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ready to chart: select K32:L35, then Insert -&gt; Bar -&gt; Clustered Bar.</t>
   </si>
   <si>
     <t xml:space="preserve">As % of quarter sales</t>
@@ -79377,7 +79386,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -79389,6 +79398,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -79884,6 +79896,15 @@
       <c r="I32" s="10" t="s">
         <v>1106</v>
       </c>
+      <c r="J32" s="9" t="s">
+        <v>1107</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>1108</v>
+      </c>
+      <c r="L32" s="10" t="s">
+        <v>1103</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
@@ -79921,6 +79942,18 @@
         <f aca="false">D33/G33</f>
         <v>348.5332</v>
       </c>
+      <c r="J33" s="3" t="str">
+        <f aca="false">"Alex – "&amp;B33</f>
+        <v>Alex – Health and beauty</v>
+      </c>
+      <c r="K33" s="3" t="str">
+        <f aca="false">INDEX($J$33:$J$35,MATCH(L33,$E$33:$E$35,0))</f>
+        <v>Giza – Home and lifestyle</v>
+      </c>
+      <c r="L33" s="20" t="n">
+        <f aca="false">LARGE($E$33:$E$35,1)</f>
+        <v>6087.627</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
@@ -79958,6 +79991,18 @@
         <f aca="false">D34/G34</f>
         <v>330.080286290323</v>
       </c>
+      <c r="J34" s="3" t="str">
+        <f aca="false">"Cairo – "&amp;B34</f>
+        <v>Cairo – Food and beverages</v>
+      </c>
+      <c r="K34" s="3" t="str">
+        <f aca="false">INDEX($J$33:$J$35,MATCH(L34,$E$33:$E$35,0))</f>
+        <v>Alex – Health and beauty</v>
+      </c>
+      <c r="L34" s="20" t="n">
+        <f aca="false">LARGE($E$33:$E$35,2)</f>
+        <v>5700.24</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
@@ -79995,19 +80040,34 @@
         <f aca="false">D35/G35</f>
         <v>347.533565217391</v>
       </c>
+      <c r="J35" s="3" t="str">
+        <f aca="false">"Giza – "&amp;B35</f>
+        <v>Giza – Home and lifestyle</v>
+      </c>
+      <c r="K35" s="3" t="str">
+        <f aca="false">INDEX($J$33:$J$35,MATCH(L35,$E$33:$E$35,0))</f>
+        <v>Cairo – Food and beverages</v>
+      </c>
+      <c r="L35" s="20" t="n">
+        <f aca="false">LARGE($E$33:$E$35,3)</f>
+        <v>5250.08925</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="E36" s="24" t="n">
         <f aca="false">SUM(E33:E35)</f>
         <v>17037.95625</v>
       </c>
+      <c r="K36" s="1" t="s">
+        <v>1110</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="E37" s="26" t="n">
         <f aca="false">E36/B5</f>
@@ -80016,12 +80076,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="23" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -80202,12 +80262,12 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="23" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -80218,21 +80278,21 @@
         <v>11</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>1090</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="B52" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$R$2:$R$1001,1)</f>
@@ -80254,7 +80314,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="B53" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$R$2:$R$1001,2)</f>
@@ -80279,7 +80339,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="B54" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$R$2:$R$1001,3)</f>
@@ -80304,12 +80364,12 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -80320,18 +80380,18 @@
         <v>11</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>1090</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="B59" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A59)</f>
@@ -80352,7 +80412,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="B60" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A60)</f>
@@ -80373,7 +80433,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B61" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A61)</f>
@@ -80394,7 +80454,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="B62" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A62)</f>
@@ -80415,7 +80475,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="B63" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A63)</f>
@@ -80436,7 +80496,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="B64" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A64)</f>
@@ -80457,7 +80517,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="B65" s="20" t="n">
         <f aca="false">SUMIFS(Data!$J$2:$J$1001,Data!$U$2:$U$1001,A65)</f>
@@ -80478,12 +80538,12 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="23" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>11</v>

</xml_diff>